<commit_message>
feat: add S1 attack branches and cross-stage highlighting
</commit_message>
<xml_diff>
--- a/docs/data/论文清单_2023-2026.xlsx
+++ b/docs/data/论文清单_2023-2026.xlsx
@@ -8,13 +8,15 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文清单" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="阶段统计" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型索引" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="检索说明" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核验摘要" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S1目标与分支" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="阶段统计" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="模型索引" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="检索说明" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核验摘要" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'论文清单'!$A$1:$N$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'论文清单'!$A$1:$R$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'S1目标与分支'!$A$1:$H$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,6 +37,10 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
   <fills count="4">
@@ -81,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -105,6 +111,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -470,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N54"/>
+  <dimension ref="A1:R54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -479,10 +494,10 @@
     <col width="6" customWidth="1" min="4" max="4"/>
     <col width="58" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="42" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
     <col width="28" customWidth="1" min="11" max="11"/>
     <col width="36" customWidth="1" min="12" max="12"/>
     <col width="38" customWidth="1" min="13" max="13"/>
@@ -522,40 +537,60 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>攻击目标代码</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>攻击目标</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>算法分支代码</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>算法分支</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>攻击接入方式</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>攻击类型</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>受影响算法/模型</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>模型信息粒度</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>实验平台/数据集</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>关键效果</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>DOI/链接</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
@@ -588,42 +623,62 @@
           <t>感知-相机 2D 检测/分类</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>相机 / 视觉传感器</t>
+        </is>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>T1a</t>
+        </is>
+      </c>
+      <c r="J2" s="9" t="inlineStr">
+        <is>
+          <t>单目 2D 检测/分类</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>物理贴片；声学信号触发相机图像畸变</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>触发式物理对抗补丁（隐藏/创建/改变）</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>YOLOv3、YOLOv5、Faster R-CNN；8 个图像分类器</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>具体型号</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>仿真 + 真实相机/车辆</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="P2" s="3" t="inlineStr">
         <is>
           <t>隐藏 88.4%、创建 91.9%、分类器改变 85.7% ASR</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>https://www.usenix.org/conference/usenixsecurity23/presentation/zhu</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="R2" s="3" t="inlineStr">
         <is>
           <t>平时良性、触发后生效；声学触发是接入关键</t>
         </is>
@@ -656,42 +711,62 @@
           <t>感知-相机 2D 检测 + 多目标跟踪（MOT）</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" s="10" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
+        <is>
+          <t>相机 / 视觉传感器</t>
+        </is>
+      </c>
+      <c r="I3" s="10" t="inlineStr">
+        <is>
+          <t>T1a</t>
+        </is>
+      </c>
+      <c r="J3" s="10" t="inlineStr">
+        <is>
+          <t>单目 2D 检测/分类</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
         <is>
           <t>打印的物理对抗补丁，贴在最优位置</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="L3" s="5" t="inlineStr">
         <is>
           <t>位置/形状劫持补丁</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="M3" s="5" t="inlineStr">
         <is>
           <t>ApoD、YOLOv3、YOLOv5、YOLOX；ApoT、BoT-SORT、ByteTrack、StrongSORT</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="N3" s="4" t="inlineStr">
         <is>
           <t>具体型号</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="O3" s="5" t="inlineStr">
         <is>
           <t>BDD、KITTI；实车</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="P3" s="5" t="inlineStr">
         <is>
           <t>平均 ASR 约 98.1%，约为最佳基线的 4 倍</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr">
+      <c r="Q3" s="5" t="inlineStr">
         <is>
           <t>10.1145/3719027.3744842</t>
         </is>
       </c>
-      <c r="N3" s="5" t="inlineStr">
+      <c r="R3" s="5" t="inlineStr">
         <is>
           <t>首次把检测+MOT 作为整体攻击面</t>
         </is>
@@ -724,42 +799,62 @@
           <t>感知-相机 2D 检测（NMS 后处理）</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>相机 / 视觉传感器</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>T1a</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>单目 2D 检测/分类</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>投影仪向场景投射对抗图案</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>物理延迟/拒绝服务（大量伪造目标）</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>相机 2D 检测器 + 多类 NMS（摘要未列具体骨干）</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>模型族</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>仿真 + 实车</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>检测目标数平均 +506%，感知延迟最高 8.1 s</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>10.1109/SP61157.2025.00236</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="R4" s="3" t="inlineStr">
         <is>
           <t>攻击面是 NMS，而非单一检测器权重</t>
         </is>
@@ -792,42 +887,62 @@
           <t>感知-单目深度估计</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>感知算法 / 数据层</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>T4c</t>
+        </is>
+      </c>
+      <c r="J5" s="10" t="inlineStr">
+        <is>
+          <t>单目深度/后门</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
         <is>
           <t>在场景中摆放普通 3D 物体，劫持透视线索；黑盒优化</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="L5" s="5" t="inlineStr">
         <is>
           <t>物理透视劫持</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="M5" s="5" t="inlineStr">
         <is>
           <t>MonoDepth2、DepthHints、ManyDepth</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="N5" s="4" t="inlineStr">
         <is>
           <t>具体型号</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="O5" s="5" t="inlineStr">
         <is>
           <t>真实场景 + 端到端 AD 仿真</t>
         </is>
       </c>
-      <c r="L5" s="5" t="inlineStr">
+      <c r="P5" s="5" t="inlineStr">
         <is>
           <t>平均深度误差增加 14 m 以上；诱发急刹、碰撞</t>
         </is>
       </c>
-      <c r="M5" s="5" t="inlineStr">
+      <c r="Q5" s="5" t="inlineStr">
         <is>
           <t>https://www.usenix.org/conference/usenixsecurity24/presentation/zheng</t>
         </is>
       </c>
-      <c r="N5" s="5" t="inlineStr">
+      <c r="R5" s="5" t="inlineStr">
         <is>
           <t>不需要贴片，普通物体即可</t>
         </is>
@@ -860,42 +975,46 @@
           <t>定位与建图-视觉 SLAM</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="9" t="inlineStr"/>
+      <c r="H6" s="9" t="inlineStr"/>
+      <c r="I6" s="9" t="inlineStr"/>
+      <c r="J6" s="9" t="inlineStr"/>
+      <c r="K6" s="3" t="inlineStr">
         <is>
           <t>道路上的低可视对抗贴片</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="L6" s="3" t="inlineStr">
         <is>
           <t>特征点/位姿攻击</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="M6" s="3" t="inlineStr">
         <is>
           <t>ORB-SLAM2、ORB-SLAM3、DynaSLAM、pl-SVO、SVO Pro</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>具体型号</t>
         </is>
       </c>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="O6" s="3" t="inlineStr">
         <is>
           <t>4Seasons 等真实/仿真序列</t>
         </is>
       </c>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="P6" s="3" t="inlineStr">
         <is>
           <t>ORB-SLAM2 误差 26.03 m，约为无攻击的 5 倍</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="Q6" s="3" t="inlineStr">
         <is>
           <t>https://www.usenix.org/conference/usenixsecurity24/presentation/chen-baodong</t>
         </is>
       </c>
-      <c r="N6" s="3" t="inlineStr">
+      <c r="R6" s="3" t="inlineStr">
         <is>
           <t>直接破坏定位与地图一致性</t>
         </is>
@@ -928,42 +1047,62 @@
           <t>感知-交通标志识别</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>相机 / 视觉传感器</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>T1b</t>
+        </is>
+      </c>
+      <c r="J7" s="10" t="inlineStr">
+        <is>
+          <t>交通标志专用视觉</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
         <is>
           <t>红外激光在标志/反射面上的不可见反射</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="L7" s="5" t="inlineStr">
         <is>
           <t>光学注入（隐藏/定向误分类）</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="M7" s="5" t="inlineStr">
         <is>
           <t>Faster R-CNN（ARTS/Mapillary）、YOLOv3、YOLOv5、GTSRB CNN</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="N7" s="4" t="inlineStr">
         <is>
           <t>具体型号</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr">
+      <c r="O7" s="5" t="inlineStr">
         <is>
           <t>真实车辆/相机、多距离</t>
         </is>
       </c>
-      <c r="L7" s="5" t="inlineStr">
+      <c r="P7" s="5" t="inlineStr">
         <is>
           <t>Faster R-CNN 达 100% ASR；YOLO 系列不稳定</t>
         </is>
       </c>
-      <c r="M7" s="5" t="inlineStr">
+      <c r="Q7" s="5" t="inlineStr">
         <is>
           <t>10.14722/ndss.2024.241053</t>
         </is>
       </c>
-      <c r="N7" s="5" t="inlineStr">
+      <c r="R7" s="5" t="inlineStr">
         <is>
           <t>利用相机红外敏感性与反射</t>
         </is>
@@ -996,42 +1135,62 @@
           <t>感知-商用交通标志识别（TSR）</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>相机 / 视觉传感器</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>T1b</t>
+        </is>
+      </c>
+      <c r="J8" s="9" t="inlineStr">
+        <is>
+          <t>交通标志专用视觉</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
         <is>
           <t>将已有物理攻击迁移到 4 款商用车型的 TSR</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="L8" s="3" t="inlineStr">
         <is>
           <t>黑盒迁移/系统级测量</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="M8" s="3" t="inlineStr">
         <is>
           <t>4 款商用 TSR 系统 + 学术 TSR 模型</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>商用系统</t>
         </is>
       </c>
-      <c r="K8" s="3" t="inlineStr">
+      <c r="O8" s="3" t="inlineStr">
         <is>
           <t>4 款美国畅销车型</t>
         </is>
       </c>
-      <c r="L8" s="3" t="inlineStr">
+      <c r="P8" s="3" t="inlineStr">
         <is>
           <t>部分功能 100% 成功，但整体泛化显著低于预期</t>
         </is>
       </c>
-      <c r="M8" s="3" t="inlineStr">
+      <c r="Q8" s="3" t="inlineStr">
         <is>
           <t>10.14722/ndss.2025.230090</t>
         </is>
       </c>
-      <c r="N8" s="3" t="inlineStr">
+      <c r="R8" s="3" t="inlineStr">
         <is>
           <t>指出商用 TSR 的空间记忆设计是主因</t>
         </is>
@@ -1064,42 +1223,62 @@
           <t>感知-交通标志/视觉识别</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>相机 / 视觉传感器</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>T1b</t>
+        </is>
+      </c>
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>交通标志专用视觉</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
         <is>
           <t>近红外（NIR）波段扰动，成本低于 50 美元</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="L9" s="5" t="inlineStr">
         <is>
           <t>定向物理逃逸</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="M9" s="5" t="inlineStr">
         <is>
           <t>YOLOv8、Faster R-CNN、GTSRB CNN、ResNet-50、ConvNeXt、Swin</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="N9" s="4" t="inlineStr">
         <is>
           <t>具体型号</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr">
+      <c r="O9" s="5" t="inlineStr">
         <is>
           <t>真实相机、多光照/距离/角度</t>
         </is>
       </c>
-      <c r="L9" s="5" t="inlineStr">
+      <c r="P9" s="5" t="inlineStr">
         <is>
           <t>ASR 较基线最高提升 20.47%</t>
         </is>
       </c>
-      <c r="M9" s="5" t="inlineStr">
+      <c r="Q9" s="5" t="inlineStr">
         <is>
           <t>10.14722/ndss.2026.231568</t>
         </is>
       </c>
-      <c r="N9" s="5" t="inlineStr">
+      <c r="R9" s="5" t="inlineStr">
         <is>
           <t>面向无红外滤光片的车载相机</t>
         </is>
@@ -1132,42 +1311,62 @@
           <t>感知-交通标志检测</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>相机 / 视觉传感器</t>
+        </is>
+      </c>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>T1b</t>
+        </is>
+      </c>
+      <c r="J10" s="9" t="inlineStr">
+        <is>
+          <t>交通标志专用视觉</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
         <is>
           <t>自然风格涂装/贴片（EOT + 视角对齐）</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="L10" s="3" t="inlineStr">
         <is>
           <t>自然化物理对抗样本</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="M10" s="3" t="inlineStr">
         <is>
           <t>交通标志检测器（ODS；摘要未列具体型号）</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>模型族</t>
         </is>
       </c>
-      <c r="K10" s="3" t="inlineStr">
+      <c r="O10" s="3" t="inlineStr">
         <is>
           <t>动态驾驶场景、多距离/角度/光照</t>
         </is>
       </c>
-      <c r="L10" s="3" t="inlineStr">
+      <c r="P10" s="3" t="inlineStr">
         <is>
           <t>多场景高 ASR，兼顾隐蔽性</t>
         </is>
       </c>
-      <c r="M10" s="3" t="inlineStr">
+      <c r="Q10" s="3" t="inlineStr">
         <is>
           <t>10.1109/TDSC.2025.3626196</t>
         </is>
       </c>
-      <c r="N10" s="3" t="inlineStr">
+      <c r="R10" s="3" t="inlineStr">
         <is>
           <t>把大扰动伪装成自然纹理</t>
         </is>
@@ -1200,42 +1399,62 @@
           <t>感知-交通标志识别（检测 + 视觉语言模型）</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>感知算法 / 数据层</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>T4c</t>
+        </is>
+      </c>
+      <c r="J11" s="10" t="inlineStr">
+        <is>
+          <t>单目深度/后门</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
         <is>
           <t>荧光墨水印刷的物理触发器；训练阶段植入后门</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="L11" s="5" t="inlineStr">
         <is>
           <t>物理后门/数据投毒</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="M11" s="5" t="inlineStr">
         <is>
           <t>Faster R-CNN、YOLOv11、LLaVA-1.5、MiniGPT-4</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr">
+      <c r="N11" s="4" t="inlineStr">
         <is>
           <t>具体型号</t>
         </is>
       </c>
-      <c r="K11" s="5" t="inlineStr">
+      <c r="O11" s="5" t="inlineStr">
         <is>
           <t>GTSRB、TSRD；真实标志</t>
         </is>
       </c>
-      <c r="L11" s="5" t="inlineStr">
+      <c r="P11" s="5" t="inlineStr">
         <is>
           <t>ASR 至少 94.23%，部分模型达 100%</t>
         </is>
       </c>
-      <c r="M11" s="5" t="inlineStr">
+      <c r="Q11" s="5" t="inlineStr">
         <is>
           <t>10.1109/TDSC.2026.3665300</t>
         </is>
       </c>
-      <c r="N11" s="5" t="inlineStr">
+      <c r="R11" s="5" t="inlineStr">
         <is>
           <t>同时攻击检测器与 VLM</t>
         </is>
@@ -1268,42 +1487,62 @@
           <t>感知-交通标志检测/限速识别</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G12" s="9" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>相机 / 视觉传感器</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>T1b</t>
+        </is>
+      </c>
+      <c r="J12" s="9" t="inlineStr">
+        <is>
+          <t>交通标志专用视觉</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
         <is>
           <t>投影仪播放高频视频帧，利用相机高速快门</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="L12" s="3" t="inlineStr">
         <is>
           <t>投影式物理对抗样本</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="M12" s="3" t="inlineStr">
         <is>
           <t>SOTA 交通标志检测器（摘要未列具体型号）</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>模型族</t>
         </is>
       </c>
-      <c r="K12" s="3" t="inlineStr">
+      <c r="O12" s="3" t="inlineStr">
         <is>
           <t>真实投影 + 相机、多条件</t>
         </is>
       </c>
-      <c r="L12" s="3" t="inlineStr">
+      <c r="P12" s="3" t="inlineStr">
         <is>
           <t>无目标 99%、有目标 90% 以上 ASR；可迁移</t>
         </is>
       </c>
-      <c r="M12" s="3" t="inlineStr">
+      <c r="Q12" s="3" t="inlineStr">
         <is>
           <t>10.1109/TIFS.2024.3422920</t>
         </is>
       </c>
-      <c r="N12" s="3" t="inlineStr">
+      <c r="R12" s="3" t="inlineStr">
         <is>
           <t>人眼几乎不可见，快门可捕获</t>
         </is>
@@ -1336,42 +1575,62 @@
           <t>感知-2D 检测/分类</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>相机 / 视觉传感器</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
+        <is>
+          <t>T1a</t>
+        </is>
+      </c>
+      <c r="J13" s="10" t="inlineStr">
+        <is>
+          <t>单目 2D 检测/分类</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
         <is>
           <t>远距离激光信号触发 + 物理贴片</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="L13" s="5" t="inlineStr">
         <is>
           <t>可控触发式补丁（隐藏/创建/定向改变）</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="M13" s="5" t="inlineStr">
         <is>
           <t>YOLOv3、YOLOv5、Faster R-CNN；VGG-13/16/19、ResNet-50/101/152、Inception-v3、MobileNet-v2</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="N13" s="4" t="inlineStr">
         <is>
           <t>具体型号</t>
         </is>
       </c>
-      <c r="K13" s="5" t="inlineStr">
+      <c r="O13" s="5" t="inlineStr">
         <is>
           <t>静止 + 移动车辆、4 款相机</t>
         </is>
       </c>
-      <c r="L13" s="5" t="inlineStr">
+      <c r="P13" s="5" t="inlineStr">
         <is>
           <t>静止 99.8/88.4/90.3%；移动 100/83.3/68.7%</t>
         </is>
       </c>
-      <c r="M13" s="5" t="inlineStr">
+      <c r="Q13" s="5" t="inlineStr">
         <is>
           <t>10.14722/ndss.2025.240026</t>
         </is>
       </c>
-      <c r="N13" s="5" t="inlineStr">
+      <c r="R13" s="5" t="inlineStr">
         <is>
           <t>解决 indiscriminate patch 问题</t>
         </is>
@@ -1404,42 +1663,46 @@
           <t>控制-无人机视觉跟踪/距离保持</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G14" s="9" t="inlineStr"/>
+      <c r="H14" s="9" t="inlineStr"/>
+      <c r="I14" s="9" t="inlineStr"/>
+      <c r="J14" s="9" t="inlineStr"/>
+      <c r="K14" s="3" t="inlineStr">
         <is>
           <t>物理对抗雨伞图案</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="L14" s="3" t="inlineStr">
         <is>
           <t>距离牵引攻击（DPA）</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="M14" s="3" t="inlineStr">
         <is>
           <t>SiamRPN-Alex/Res/Mobile、MixFormer；SORT、UCMCTrack；DJI、HoverAir</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="N14" s="2" t="inlineStr">
         <is>
           <t>具体型号</t>
         </is>
       </c>
-      <c r="K14" s="3" t="inlineStr">
+      <c r="O14" s="3" t="inlineStr">
         <is>
           <t>仿真 + 商业无人机实飞</t>
         </is>
       </c>
-      <c r="L14" s="3" t="inlineStr">
+      <c r="P14" s="3" t="inlineStr">
         <is>
           <t>9 m 内 100% 捕获；6 m 内 100% DoubleStar</t>
         </is>
       </c>
-      <c r="M14" s="3" t="inlineStr">
+      <c r="Q14" s="3" t="inlineStr">
         <is>
           <t>10.14722/ndss.2026.230904</t>
         </is>
       </c>
-      <c r="N14" s="3" t="inlineStr">
+      <c r="R14" s="3" t="inlineStr">
         <is>
           <t>从感知欺骗升级为物理捕获</t>
         </is>
@@ -1472,42 +1735,46 @@
           <t>控制-云台 + 感知-视觉跟踪</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="G15" s="10" t="inlineStr"/>
+      <c r="H15" s="10" t="inlineStr"/>
+      <c r="I15" s="10" t="inlineStr"/>
+      <c r="J15" s="10" t="inlineStr"/>
+      <c r="K15" s="5" t="inlineStr">
         <is>
           <t>声学波形注入，激发云台谐振</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="L15" s="5" t="inlineStr">
         <is>
           <t>云台视角漂移/目标切换</t>
         </is>
       </c>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="M15" s="5" t="inlineStr">
         <is>
           <t>SiamRPN、SORT、KCF、DaSiamRPN、UCMCTrack；2 款商用云台</t>
         </is>
       </c>
-      <c r="J15" s="4" t="inlineStr">
+      <c r="N15" s="4" t="inlineStr">
         <is>
           <t>具体型号</t>
         </is>
       </c>
-      <c r="K15" s="5" t="inlineStr">
+      <c r="O15" s="5" t="inlineStr">
         <is>
           <t>仿真 + 台架 + 商业无人机实飞</t>
         </is>
       </c>
-      <c r="L15" s="5" t="inlineStr">
+      <c r="P15" s="5" t="inlineStr">
         <is>
           <t>仿真 93.6%，真实 95.5% 目标切换成功率</t>
         </is>
       </c>
-      <c r="M15" s="5" t="inlineStr">
+      <c r="Q15" s="5" t="inlineStr">
         <is>
           <t>10.1109/SP63933.2026.00129</t>
         </is>
       </c>
-      <c r="N15" s="5" t="inlineStr">
+      <c r="R15" s="5" t="inlineStr">
         <is>
           <t>跨声学-视觉域，黑盒</t>
         </is>
@@ -1540,42 +1807,62 @@
           <t>感知-视觉单目标跟踪</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>感知算法 / 数据层</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>T4b</t>
+        </is>
+      </c>
+      <c r="J16" s="9" t="inlineStr">
+        <is>
+          <t>视觉单目标跟踪</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
         <is>
           <t>数字扰动（连续视频帧）</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="L16" s="3" t="inlineStr">
         <is>
           <t>多策略轨迹劫持</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="M16" s="3" t="inlineStr">
         <is>
           <t>视觉跟踪器（摘要未列具体型号）</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>模型族</t>
         </is>
       </c>
-      <c r="K16" s="3" t="inlineStr">
+      <c r="O16" s="3" t="inlineStr">
         <is>
           <t>多个公开跟踪基准</t>
         </is>
       </c>
-      <c r="L16" s="3" t="inlineStr">
+      <c r="P16" s="3" t="inlineStr">
         <is>
           <t>长期欺骗与多目标场景优于 SOTA</t>
         </is>
       </c>
-      <c r="M16" s="3" t="inlineStr">
+      <c r="Q16" s="3" t="inlineStr">
         <is>
           <t>10.1109/TDSC.2025.3582615</t>
         </is>
       </c>
-      <c r="N16" s="3" t="inlineStr">
+      <c r="R16" s="3" t="inlineStr">
         <is>
           <t>强调持续性与隐蔽性</t>
         </is>
@@ -1608,42 +1895,62 @@
           <t>感知-视觉单目标跟踪</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>感知算法 / 数据层</t>
+        </is>
+      </c>
+      <c r="I17" s="10" t="inlineStr">
+        <is>
+          <t>T4b</t>
+        </is>
+      </c>
+      <c r="J17" s="10" t="inlineStr">
+        <is>
+          <t>视觉单目标跟踪</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
         <is>
           <t>数字扰动（源图像特征级）</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="L17" s="5" t="inlineStr">
         <is>
           <t>特征级通用攻击</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
+      <c r="M17" s="5" t="inlineStr">
         <is>
           <t>DCF、Siamese、Transformer 三类跟踪器</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr">
+      <c r="N17" s="4" t="inlineStr">
         <is>
           <t>模型族（三类）</t>
         </is>
       </c>
-      <c r="K17" s="5" t="inlineStr">
+      <c r="O17" s="5" t="inlineStr">
         <is>
           <t>OTB100、UAV123、LaSOT、TLP</t>
         </is>
       </c>
-      <c r="L17" s="5" t="inlineStr">
+      <c r="P17" s="5" t="inlineStr">
         <is>
           <t>可插拔；与决策级攻击可联合优化</t>
         </is>
       </c>
-      <c r="M17" s="5" t="inlineStr">
+      <c r="Q17" s="5" t="inlineStr">
         <is>
           <t>10.1109/TIFS.2023.3331899</t>
         </is>
       </c>
-      <c r="N17" s="5" t="inlineStr">
+      <c r="R17" s="5" t="inlineStr">
         <is>
           <t>不依赖具体跟踪器输出形式</t>
         </is>
@@ -1676,42 +1983,62 @@
           <t>感知-LiDAR 3D 检测</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>LiDAR / 点云传感器</t>
+        </is>
+      </c>
+      <c r="I18" s="9" t="inlineStr">
+        <is>
+          <t>T2a</t>
+        </is>
+      </c>
+      <c r="J18" s="9" t="inlineStr">
+        <is>
+          <t>LiDAR 3D 检测</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
         <is>
           <t>激光注入伪造点云（最高 4200 点）</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
+      <c r="L18" s="3" t="inlineStr">
         <is>
           <t>物理点云注入（隐藏/创建）</t>
         </is>
       </c>
-      <c r="I18" s="3" t="inlineStr">
+      <c r="M18" s="3" t="inlineStr">
         <is>
           <t>3 个 LiDAR 3D 检测器（摘要未列名）；2 款商用 LiDAR</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>模型族</t>
         </is>
       </c>
-      <c r="K18" s="3" t="inlineStr">
+      <c r="O18" s="3" t="inlineStr">
         <is>
           <t>真实 LiDAR + 车辆</t>
         </is>
       </c>
-      <c r="L18" s="3" t="inlineStr">
+      <c r="P18" s="3" t="inlineStr">
         <is>
           <t>4 类攻击（naive/record/opt-hide/opt-create）均有效</t>
         </is>
       </c>
-      <c r="M18" s="3" t="inlineStr">
+      <c r="Q18" s="3" t="inlineStr">
         <is>
           <t>10.1109/SP46215.2023.10179458</t>
         </is>
       </c>
-      <c r="N18" s="3" t="inlineStr">
+      <c r="R18" s="3" t="inlineStr">
         <is>
           <t>可测量 victim LiDAR 扫描周期</t>
         </is>
@@ -1744,42 +2071,62 @@
           <t>感知-LiDAR 3D 检测</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>LiDAR / 点云传感器</t>
+        </is>
+      </c>
+      <c r="I19" s="10" t="inlineStr">
+        <is>
+          <t>T2a</t>
+        </is>
+      </c>
+      <c r="J19" s="10" t="inlineStr">
+        <is>
+          <t>LiDAR 3D 检测</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
         <is>
           <t>3D 打印对抗饰品 + 物体重建</t>
         </is>
       </c>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="L19" s="5" t="inlineStr">
         <is>
           <t>物理对抗物体</t>
         </is>
       </c>
-      <c r="I19" s="5" t="inlineStr">
+      <c r="M19" s="5" t="inlineStr">
         <is>
           <t>PointPillars、PointRCNN；Apollo 7.0</t>
         </is>
       </c>
-      <c r="J19" s="4" t="inlineStr">
+      <c r="N19" s="4" t="inlineStr">
         <is>
           <t>具体型号</t>
         </is>
       </c>
-      <c r="K19" s="5" t="inlineStr">
+      <c r="O19" s="5" t="inlineStr">
         <is>
           <t>静态 + 20 m 动态实车</t>
         </is>
       </c>
-      <c r="L19" s="5" t="inlineStr">
+      <c r="P19" s="5" t="inlineStr">
         <is>
           <t>动态 100% ASR；存活率 +38%（PointPillars）/+22%（PointRCNN）</t>
         </is>
       </c>
-      <c r="M19" s="5" t="inlineStr">
+      <c r="Q19" s="5" t="inlineStr">
         <is>
           <t>https://www.usenix.org/conference/usenixsecurity24/presentation/zhu-shenchen</t>
         </is>
       </c>
-      <c r="N19" s="5" t="inlineStr">
+      <c r="R19" s="5" t="inlineStr">
         <is>
           <t>解决物理世界形状/视角变化</t>
         </is>
@@ -1812,42 +2159,62 @@
           <t>感知-LiDAR 3D 检测</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t>LiDAR / 点云传感器</t>
+        </is>
+      </c>
+      <c r="I20" s="9" t="inlineStr">
+        <is>
+          <t>T2a</t>
+        </is>
+      </c>
+      <c r="J20" s="9" t="inlineStr">
+        <is>
+          <t>LiDAR 3D 检测</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
         <is>
           <t>反光镜片制造对抗阴影，删除点云</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
+      <c r="L20" s="3" t="inlineStr">
         <is>
           <t>物理点云移除</t>
         </is>
       </c>
-      <c r="I20" s="3" t="inlineStr">
+      <c r="M20" s="3" t="inlineStr">
         <is>
           <t>PointPillars、SECOND-IoU、PointRCNN</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>具体型号</t>
         </is>
       </c>
-      <c r="K20" s="3" t="inlineStr">
+      <c r="O20" s="3" t="inlineStr">
         <is>
           <t>真实 LiDAR、1–23 m</t>
         </is>
       </c>
-      <c r="L20" s="3" t="inlineStr">
+      <c r="P20" s="3" t="inlineStr">
         <is>
           <t>10 m 处 PointPillars 100%、SECOND-IoU 98%</t>
         </is>
       </c>
-      <c r="M20" s="3" t="inlineStr">
+      <c r="Q20" s="3" t="inlineStr">
         <is>
           <t>https://www.usenix.org/conference/usenixsecurity25/presentation/kobayashi</t>
         </is>
       </c>
-      <c r="N20" s="3" t="inlineStr">
+      <c r="R20" s="3" t="inlineStr">
         <is>
           <t>同时提出检测防御</t>
         </is>
@@ -1880,42 +2247,62 @@
           <t>感知-LiDAR/深度相机</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="G21" s="10" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="H21" s="10" t="inlineStr">
+        <is>
+          <t>LiDAR / 点云传感器</t>
+        </is>
+      </c>
+      <c r="I21" s="10" t="inlineStr">
+        <is>
+          <t>T2b</t>
+        </is>
+      </c>
+      <c r="J21" s="10" t="inlineStr">
+        <is>
+          <t>点云欺骗/闭环验证</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
         <is>
           <t>红外染料涂层改变反射率，诱发测距 walk error</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="L21" s="5" t="inlineStr">
         <is>
           <t>物理反射率欺骗</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr">
+      <c r="M21" s="5" t="inlineStr">
         <is>
           <t>点云分类、分割、检测下游模型（摘要未列名）</t>
         </is>
       </c>
-      <c r="J21" s="4" t="inlineStr">
+      <c r="N21" s="4" t="inlineStr">
         <is>
           <t>模型族</t>
         </is>
       </c>
-      <c r="K21" s="5" t="inlineStr">
+      <c r="O21" s="5" t="inlineStr">
         <is>
           <t>LiDAR + 深度相机</t>
         </is>
       </c>
-      <c r="L21" s="5" t="inlineStr">
+      <c r="P21" s="5" t="inlineStr">
         <is>
           <t>定向误分类、误分割、检测失败</t>
         </is>
       </c>
-      <c r="M21" s="5" t="inlineStr">
+      <c r="Q21" s="5" t="inlineStr">
         <is>
           <t>10.1109/SP63933.2026.00183</t>
         </is>
       </c>
-      <c r="N21" s="5" t="inlineStr">
+      <c r="R21" s="5" t="inlineStr">
         <is>
           <t>可见光下几乎不可见</t>
         </is>
@@ -1948,42 +2335,62 @@
           <t>感知-LiDAR 3D 检测</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>LiDAR / 点云传感器</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>T2a</t>
+        </is>
+      </c>
+      <c r="J22" s="9" t="inlineStr">
+        <is>
+          <t>LiDAR 3D 检测</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
         <is>
           <t>高频激光移除/点云删除</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr">
+      <c r="L22" s="3" t="inlineStr">
         <is>
           <t>物理点云移除（HFR/PRA）</t>
         </is>
       </c>
-      <c r="I22" s="3" t="inlineStr">
+      <c r="M22" s="3" t="inlineStr">
         <is>
           <t>PointPillars、SECOND、Part-A2、3DSSD、PV-RCNN；Apollo</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="N22" s="2" t="inlineStr">
         <is>
           <t>具体型号</t>
         </is>
       </c>
-      <c r="K22" s="3" t="inlineStr">
+      <c r="O22" s="3" t="inlineStr">
         <is>
           <t>真实 LiDAR + Apollo</t>
         </is>
       </c>
-      <c r="L22" s="3" t="inlineStr">
+      <c r="P22" s="3" t="inlineStr">
         <is>
           <t>5 辆前车连续 10 s 以上 100% 消失</t>
         </is>
       </c>
-      <c r="M22" s="3" t="inlineStr">
+      <c r="Q22" s="3" t="inlineStr">
         <is>
           <t>https://www.usenix.org/conference/usenixsecurity23/presentation/cao</t>
         </is>
       </c>
-      <c r="N22" s="3" t="inlineStr">
+      <c r="R22" s="3" t="inlineStr">
         <is>
           <t>从注入转向删除</t>
         </is>
@@ -2016,42 +2423,62 @@
           <t>感知-LiDAR 3D 检测</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="G23" s="10" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="H23" s="10" t="inlineStr">
+        <is>
+          <t>LiDAR / 点云传感器</t>
+        </is>
+      </c>
+      <c r="I23" s="10" t="inlineStr">
+        <is>
+          <t>T2a</t>
+        </is>
+      </c>
+      <c r="J23" s="10" t="inlineStr">
+        <is>
+          <t>LiDAR 3D 检测</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
         <is>
           <t>激光注入/点云伪造</t>
         </is>
       </c>
-      <c r="H23" s="5" t="inlineStr">
+      <c r="L23" s="5" t="inlineStr">
         <is>
           <t>点云伪造/移除</t>
         </is>
       </c>
-      <c r="I23" s="5" t="inlineStr">
+      <c r="M23" s="5" t="inlineStr">
         <is>
           <t>PointPillars、SECOND、Part-A2、3DSSD、PV-RCNN；5 个训练数据集</t>
         </is>
       </c>
-      <c r="J23" s="4" t="inlineStr">
+      <c r="N23" s="4" t="inlineStr">
         <is>
           <t>具体型号</t>
         </is>
       </c>
-      <c r="K23" s="5" t="inlineStr">
+      <c r="O23" s="5" t="inlineStr">
         <is>
           <t>多款 LiDAR、真实道路</t>
         </is>
       </c>
-      <c r="L23" s="5" t="inlineStr">
+      <c r="P23" s="5" t="inlineStr">
         <is>
           <t>多模型高 ASR；时序随机化可降低</t>
         </is>
       </c>
-      <c r="M23" s="5" t="inlineStr">
+      <c r="Q23" s="5" t="inlineStr">
         <is>
           <t>10.14722/ndss.2024.23350</t>
         </is>
       </c>
-      <c r="N23" s="5" t="inlineStr">
+      <c r="R23" s="5" t="inlineStr">
         <is>
           <t>系统评估新一代 LiDAR 的假设</t>
         </is>
@@ -2084,42 +2511,62 @@
           <t>感知-LiDAR + 规划控制闭环</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="H24" s="9" t="inlineStr">
+        <is>
+          <t>LiDAR / 点云传感器</t>
+        </is>
+      </c>
+      <c r="I24" s="9" t="inlineStr">
+        <is>
+          <t>T2b</t>
+        </is>
+      </c>
+      <c r="J24" s="9" t="inlineStr">
+        <is>
+          <t>点云欺骗/闭环验证</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
         <is>
           <t>高速/远距离激光注入</t>
         </is>
       </c>
-      <c r="H24" s="3" t="inlineStr">
+      <c r="L24" s="3" t="inlineStr">
         <is>
           <t>长时点云欺骗</t>
         </is>
       </c>
-      <c r="I24" s="3" t="inlineStr">
+      <c r="M24" s="3" t="inlineStr">
         <is>
           <t>YOLOv5（瞄准）、Autoware（闭环）</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr">
+      <c r="N24" s="2" t="inlineStr">
         <is>
           <t>具体型号</t>
         </is>
       </c>
-      <c r="K24" s="3" t="inlineStr">
+      <c r="O24" s="3" t="inlineStr">
         <is>
           <t>真实道路、高速场景</t>
         </is>
       </c>
-      <c r="L24" s="3" t="inlineStr">
+      <c r="P24" s="3" t="inlineStr">
         <is>
           <t>持续 100 s 以上；高速远距离可行</t>
         </is>
       </c>
-      <c r="M24" s="3" t="inlineStr">
+      <c r="Q24" s="3" t="inlineStr">
         <is>
           <t>10.14722/ndss.2025.230628</t>
         </is>
       </c>
-      <c r="N24" s="3" t="inlineStr">
+      <c r="R24" s="3" t="inlineStr">
         <is>
           <t>首次高速远距离闭环评估</t>
         </is>
@@ -2152,42 +2599,62 @@
           <t>感知-相机（车辆外观）</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
+      <c r="G25" s="10" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="H25" s="10" t="inlineStr">
+        <is>
+          <t>相机 / 视觉传感器</t>
+        </is>
+      </c>
+      <c r="I25" s="10" t="inlineStr">
+        <is>
+          <t>T1c</t>
+        </is>
+      </c>
+      <c r="J25" s="10" t="inlineStr">
+        <is>
+          <t>多视角/机器人视觉</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
         <is>
           <t>可打印的 3D Gaussian 对抗车衣</t>
         </is>
       </c>
-      <c r="H25" s="5" t="inlineStr">
+      <c r="L25" s="5" t="inlineStr">
         <is>
           <t>多视角物理对抗纹理</t>
         </is>
       </c>
-      <c r="I25" s="5" t="inlineStr">
+      <c r="M25" s="5" t="inlineStr">
         <is>
           <t>多个现代相机检测器（摘要未列名）</t>
         </is>
       </c>
-      <c r="J25" s="4" t="inlineStr">
+      <c r="N25" s="4" t="inlineStr">
         <is>
           <t>模型族</t>
         </is>
       </c>
-      <c r="K25" s="5" t="inlineStr">
+      <c r="O25" s="5" t="inlineStr">
         <is>
           <t>CARLA + 微型车实物</t>
         </is>
       </c>
-      <c r="L25" s="5" t="inlineStr">
+      <c r="P25" s="5" t="inlineStr">
         <is>
           <t>多视角检测置信度/AP 显著下降</t>
         </is>
       </c>
-      <c r="M25" s="5" t="inlineStr">
+      <c r="Q25" s="5" t="inlineStr">
         <is>
           <t>10.1109/TIFS.2026.3729511</t>
         </is>
       </c>
-      <c r="N25" s="5" t="inlineStr">
+      <c r="R25" s="5" t="inlineStr">
         <is>
           <t>保持车辆几何形状，仅改纹理</t>
         </is>
@@ -2220,42 +2687,62 @@
           <t>感知-视觉 + LiDAR 3D 检测</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr">
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="H26" s="9" t="inlineStr">
+        <is>
+          <t>LiDAR / 点云传感器</t>
+        </is>
+      </c>
+      <c r="I26" s="9" t="inlineStr">
+        <is>
+          <t>T2c</t>
+        </is>
+      </c>
+      <c r="J26" s="9" t="inlineStr">
+        <is>
+          <t>跨模态/多传感器融合</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
         <is>
           <t>NeRF 生成可制造的 3D 对抗网格</t>
         </is>
       </c>
-      <c r="H26" s="3" t="inlineStr">
+      <c r="L26" s="3" t="inlineStr">
         <is>
           <t>跨模态对抗物体</t>
         </is>
       </c>
-      <c r="I26" s="3" t="inlineStr">
+      <c r="M26" s="3" t="inlineStr">
         <is>
           <t>视觉与 LiDAR 3D 检测器（摘要未列名）</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="N26" s="2" t="inlineStr">
         <is>
           <t>模型族</t>
         </is>
       </c>
-      <c r="K26" s="3" t="inlineStr">
+      <c r="O26" s="3" t="inlineStr">
         <is>
           <t>多视角、仿真/实物</t>
         </is>
       </c>
-      <c r="L26" s="3" t="inlineStr">
+      <c r="P26" s="3" t="inlineStr">
         <is>
           <t>多视角下降低 3D 检测精度</t>
         </is>
       </c>
-      <c r="M26" s="3" t="inlineStr">
+      <c r="Q26" s="3" t="inlineStr">
         <is>
           <t>10.1109/TIFS.2025.3609180</t>
         </is>
       </c>
-      <c r="N26" s="3" t="inlineStr">
+      <c r="R26" s="3" t="inlineStr">
         <is>
           <t>同时针对视觉与 LiDAR</t>
         </is>
@@ -2288,42 +2775,62 @@
           <t>感知-LiDAR 预处理</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr">
+      <c r="G27" s="10" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="H27" s="10" t="inlineStr">
+        <is>
+          <t>感知算法 / 数据层</t>
+        </is>
+      </c>
+      <c r="I27" s="10" t="inlineStr">
+        <is>
+          <t>T4a</t>
+        </is>
+      </c>
+      <c r="J27" s="10" t="inlineStr">
+        <is>
+          <t>点云分类与预处理</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr">
         <is>
           <t>针对点云预处理/滤波器的对抗雾</t>
         </is>
       </c>
-      <c r="H27" s="5" t="inlineStr">
+      <c r="L27" s="5" t="inlineStr">
         <is>
           <t>预处理层攻击</t>
         </is>
       </c>
-      <c r="I27" s="5" t="inlineStr">
+      <c r="M27" s="5" t="inlineStr">
         <is>
           <t>LiDAR 点云预处理滤波器（摘要未公开）</t>
         </is>
       </c>
-      <c r="J27" s="4" t="inlineStr">
+      <c r="N27" s="4" t="inlineStr">
         <is>
           <t>未披露</t>
         </is>
       </c>
-      <c r="K27" s="5" t="inlineStr">
+      <c r="O27" s="5" t="inlineStr">
         <is>
           <t>LiDAR 点云</t>
         </is>
       </c>
-      <c r="L27" s="5" t="inlineStr">
+      <c r="P27" s="5" t="inlineStr">
         <is>
           <t>利用滤波器漏洞（公开摘要不足）</t>
         </is>
       </c>
-      <c r="M27" s="5" t="inlineStr">
+      <c r="Q27" s="5" t="inlineStr">
         <is>
           <t>10.1145/3708821.3733904</t>
         </is>
       </c>
-      <c r="N27" s="5" t="inlineStr">
+      <c r="R27" s="5" t="inlineStr">
         <is>
           <t>把攻击面前移到预处理</t>
         </is>
@@ -2356,42 +2863,62 @@
           <t>感知-点云分类</t>
         </is>
       </c>
-      <c r="G28" s="3" t="inlineStr">
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="H28" s="9" t="inlineStr">
+        <is>
+          <t>感知算法 / 数据层</t>
+        </is>
+      </c>
+      <c r="I28" s="9" t="inlineStr">
+        <is>
+          <t>T4a</t>
+        </is>
+      </c>
+      <c r="J28" s="9" t="inlineStr">
+        <is>
+          <t>点云分类与预处理</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
         <is>
           <t>数字点云形变（cage-based）</t>
         </is>
       </c>
-      <c r="H28" s="3" t="inlineStr">
+      <c r="L28" s="3" t="inlineStr">
         <is>
           <t>语义一致对抗形变</t>
         </is>
       </c>
-      <c r="I28" s="3" t="inlineStr">
+      <c r="M28" s="3" t="inlineStr">
         <is>
           <t>点云分类器；ModelNet40、ShapeNet-Part、ScanObjectNN</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr">
+      <c r="N28" s="2" t="inlineStr">
         <is>
           <t>模型族</t>
         </is>
       </c>
-      <c r="K28" s="3" t="inlineStr">
+      <c r="O28" s="3" t="inlineStr">
         <is>
           <t>三个点云基准</t>
         </is>
       </c>
-      <c r="L28" s="3" t="inlineStr">
+      <c r="P28" s="3" t="inlineStr">
         <is>
           <t>高 ASR，几何失真低，抗多种防御</t>
         </is>
       </c>
-      <c r="M28" s="3" t="inlineStr">
+      <c r="Q28" s="3" t="inlineStr">
         <is>
           <t>10.1109/TIFS.2026.3696199</t>
         </is>
       </c>
-      <c r="N28" s="3" t="inlineStr">
+      <c r="R28" s="3" t="inlineStr">
         <is>
           <t>强调语义一致性</t>
         </is>
@@ -2424,42 +2951,62 @@
           <t>感知-点云分类</t>
         </is>
       </c>
-      <c r="G29" s="5" t="inlineStr">
+      <c r="G29" s="10" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="H29" s="10" t="inlineStr">
+        <is>
+          <t>感知算法 / 数据层</t>
+        </is>
+      </c>
+      <c r="I29" s="10" t="inlineStr">
+        <is>
+          <t>T4a</t>
+        </is>
+      </c>
+      <c r="J29" s="10" t="inlineStr">
+        <is>
+          <t>点云分类与预处理</t>
+        </is>
+      </c>
+      <c r="K29" s="5" t="inlineStr">
         <is>
           <t>仅可查询预测标签（hard-label 黑盒）</t>
         </is>
       </c>
-      <c r="H29" s="5" t="inlineStr">
+      <c r="L29" s="5" t="inlineStr">
         <is>
           <t>硬标签黑盒攻击</t>
         </is>
       </c>
-      <c r="I29" s="5" t="inlineStr">
+      <c r="M29" s="5" t="inlineStr">
         <is>
           <t>点云分类器（摘要未列名）</t>
         </is>
       </c>
-      <c r="J29" s="4" t="inlineStr">
+      <c r="N29" s="4" t="inlineStr">
         <is>
           <t>模型族</t>
         </is>
       </c>
-      <c r="K29" s="5" t="inlineStr">
+      <c r="O29" s="5" t="inlineStr">
         <is>
           <t>3D 点云基准</t>
         </is>
       </c>
-      <c r="L29" s="5" t="inlineStr">
+      <c r="P29" s="5" t="inlineStr">
         <is>
           <t>查询高效、扰动小</t>
         </is>
       </c>
-      <c r="M29" s="5" t="inlineStr">
+      <c r="Q29" s="5" t="inlineStr">
         <is>
           <t>10.1109/TDSC.2026.3694723</t>
         </is>
       </c>
-      <c r="N29" s="5" t="inlineStr">
+      <c r="R29" s="5" t="inlineStr">
         <is>
           <t>更贴近真实部署威胁模型</t>
         </is>
@@ -2492,42 +3039,62 @@
           <t>感知-点云分类（训练阶段）</t>
         </is>
       </c>
-      <c r="G30" s="3" t="inlineStr">
+      <c r="G30" s="9" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="H30" s="9" t="inlineStr">
+        <is>
+          <t>感知算法 / 数据层</t>
+        </is>
+      </c>
+      <c r="I30" s="9" t="inlineStr">
+        <is>
+          <t>T4a</t>
+        </is>
+      </c>
+      <c r="J30" s="9" t="inlineStr">
+        <is>
+          <t>点云分类与预处理</t>
+        </is>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
         <is>
           <t>训练数据投毒 + 触发器</t>
         </is>
       </c>
-      <c r="H30" s="3" t="inlineStr">
+      <c r="L30" s="3" t="inlineStr">
         <is>
           <t>抗腐蚀后门</t>
         </is>
       </c>
-      <c r="I30" s="3" t="inlineStr">
+      <c r="M30" s="3" t="inlineStr">
         <is>
           <t>PointNet、PointNet++</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr">
+      <c r="N30" s="2" t="inlineStr">
         <is>
           <t>具体型号</t>
         </is>
       </c>
-      <c r="K30" s="3" t="inlineStr">
+      <c r="O30" s="3" t="inlineStr">
         <is>
           <t>点云分类基准、多种腐蚀</t>
         </is>
       </c>
-      <c r="L30" s="3" t="inlineStr">
+      <c r="P30" s="3" t="inlineStr">
         <is>
           <t>高 ASR，抗点云腐蚀</t>
         </is>
       </c>
-      <c r="M30" s="3" t="inlineStr">
+      <c r="Q30" s="3" t="inlineStr">
         <is>
           <t>10.1109/TIFS.2025.3575274</t>
         </is>
       </c>
-      <c r="N30" s="3" t="inlineStr">
+      <c r="R30" s="3" t="inlineStr">
         <is>
           <t>利用 affinity 类别稳定特征</t>
         </is>
@@ -2560,42 +3127,62 @@
           <t>感知-2D 目标检测</t>
         </is>
       </c>
-      <c r="G31" s="5" t="inlineStr">
+      <c r="G31" s="10" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="H31" s="10" t="inlineStr">
+        <is>
+          <t>相机 / 视觉传感器</t>
+        </is>
+      </c>
+      <c r="I31" s="10" t="inlineStr">
+        <is>
+          <t>T1a</t>
+        </is>
+      </c>
+      <c r="J31" s="10" t="inlineStr">
+        <is>
+          <t>单目 2D 检测/分类</t>
+        </is>
+      </c>
+      <c r="K31" s="5" t="inlineStr">
         <is>
           <t>物理贴片（多尺度 + 模糊模拟）</t>
         </is>
       </c>
-      <c r="H31" s="5" t="inlineStr">
+      <c r="L31" s="5" t="inlineStr">
         <is>
           <t>多尺度鲁棒补丁</t>
         </is>
       </c>
-      <c r="I31" s="5" t="inlineStr">
+      <c r="M31" s="5" t="inlineStr">
         <is>
           <t>多个 2D 目标检测器（摘要未列名）</t>
         </is>
       </c>
-      <c r="J31" s="4" t="inlineStr">
+      <c r="N31" s="4" t="inlineStr">
         <is>
           <t>模型族</t>
         </is>
       </c>
-      <c r="K31" s="5" t="inlineStr">
+      <c r="O31" s="5" t="inlineStr">
         <is>
           <t>数字 + 仿真 + 物理</t>
         </is>
       </c>
-      <c r="L31" s="5" t="inlineStr">
+      <c r="P31" s="5" t="inlineStr">
         <is>
           <t>距离/模糊/遮挡下保持高 ASR</t>
         </is>
       </c>
-      <c r="M31" s="5" t="inlineStr">
+      <c r="Q31" s="5" t="inlineStr">
         <is>
           <t>10.1109/TDSC.2026.3681111</t>
         </is>
       </c>
-      <c r="N31" s="5" t="inlineStr">
+      <c r="R31" s="5" t="inlineStr">
         <is>
           <t>用自相似性保持多尺度效果</t>
         </is>
@@ -2628,42 +3215,62 @@
           <t>感知-mmWave 雷达检测</t>
         </is>
       </c>
-      <c r="G32" s="3" t="inlineStr">
+      <c r="G32" s="9" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="H32" s="9" t="inlineStr">
+        <is>
+          <t>毫米波雷达传感器</t>
+        </is>
+      </c>
+      <c r="I32" s="9" t="inlineStr">
+        <is>
+          <t>T3a</t>
+        </is>
+      </c>
+      <c r="J32" s="9" t="inlineStr">
+        <is>
+          <t>学习型雷达检测</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
         <is>
           <t>低成本 3D 打印 + 金属箔被动反射物</t>
         </is>
       </c>
-      <c r="H32" s="3" t="inlineStr">
+      <c r="L32" s="3" t="inlineStr">
         <is>
           <t>被动反射对抗物体</t>
         </is>
       </c>
-      <c r="I32" s="3" t="inlineStr">
+      <c r="M32" s="3" t="inlineStr">
         <is>
           <t>DNN 雷达目标检测模型（摘要未列名）</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr">
+      <c r="N32" s="2" t="inlineStr">
         <is>
           <t>模型族</t>
         </is>
       </c>
-      <c r="K32" s="3" t="inlineStr">
+      <c r="O32" s="3" t="inlineStr">
         <is>
           <t>真实 mmWave 雷达</t>
         </is>
       </c>
-      <c r="L32" s="3" t="inlineStr">
+      <c r="P32" s="3" t="inlineStr">
         <is>
           <t>无需同步、低成本，可欺骗 DNN 检测</t>
         </is>
       </c>
-      <c r="M32" s="3" t="inlineStr">
+      <c r="Q32" s="3" t="inlineStr">
         <is>
           <t>10.1145/3576915.3616661</t>
         </is>
       </c>
-      <c r="N32" s="3" t="inlineStr">
+      <c r="R32" s="3" t="inlineStr">
         <is>
           <t>不主动发射信号</t>
         </is>
@@ -2696,42 +3303,62 @@
           <t>感知-mmWave 雷达</t>
         </is>
       </c>
-      <c r="G33" s="5" t="inlineStr">
+      <c r="G33" s="10" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="H33" s="10" t="inlineStr">
+        <is>
+          <t>毫米波雷达传感器</t>
+        </is>
+      </c>
+      <c r="I33" s="10" t="inlineStr">
+        <is>
+          <t>T3b</t>
+        </is>
+      </c>
+      <c r="J33" s="10" t="inlineStr">
+        <is>
+          <t>FMCW 信号层</t>
+        </is>
+      </c>
+      <c r="K33" s="5" t="inlineStr">
         <is>
           <t>软件定义无线电 + 实时参数估计</t>
         </is>
       </c>
-      <c r="H33" s="5" t="inlineStr">
+      <c r="L33" s="5" t="inlineStr">
         <is>
           <t>黑盒物理层欺骗（增/删/移）</t>
         </is>
       </c>
-      <c r="I33" s="5" t="inlineStr">
+      <c r="M33" s="5" t="inlineStr">
         <is>
           <t>FMCW 雷达点云（非 DNN）</t>
         </is>
       </c>
-      <c r="J33" s="4" t="inlineStr">
+      <c r="N33" s="4" t="inlineStr">
         <is>
           <t>信号处理</t>
         </is>
       </c>
-      <c r="K33" s="5" t="inlineStr">
+      <c r="O33" s="5" t="inlineStr">
         <is>
           <t>真实雷达 + SDR 原型</t>
         </is>
       </c>
-      <c r="L33" s="5" t="inlineStr">
+      <c r="P33" s="5" t="inlineStr">
         <is>
           <t>可添加、删除、平移目标检测</t>
         </is>
       </c>
-      <c r="M33" s="5" t="inlineStr">
+      <c r="Q33" s="5" t="inlineStr">
         <is>
           <t>10.14722/ndss.2024.24153</t>
         </is>
       </c>
-      <c r="N33" s="5" t="inlineStr">
+      <c r="R33" s="5" t="inlineStr">
         <is>
           <t>无需预先知道雷达配置</t>
         </is>
@@ -2764,42 +3391,62 @@
           <t>感知-mmWave 雷达</t>
         </is>
       </c>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="G34" s="9" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="H34" s="9" t="inlineStr">
+        <is>
+          <t>毫米波雷达传感器</t>
+        </is>
+      </c>
+      <c r="I34" s="9" t="inlineStr">
+        <is>
+          <t>T3b</t>
+        </is>
+      </c>
+      <c r="J34" s="9" t="inlineStr">
+        <is>
+          <t>FMCW 信号层</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
         <is>
           <t>反射阵列（reflect array）调制</t>
         </is>
       </c>
-      <c r="H34" s="3" t="inlineStr">
+      <c r="L34" s="3" t="inlineStr">
         <is>
           <t>无同步距离/速度欺骗</t>
         </is>
       </c>
-      <c r="I34" s="3" t="inlineStr">
+      <c r="M34" s="3" t="inlineStr">
         <is>
           <t>FMCW 雷达信号处理</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr">
+      <c r="N34" s="2" t="inlineStr">
         <is>
           <t>信号处理</t>
         </is>
       </c>
-      <c r="K34" s="3" t="inlineStr">
+      <c r="O34" s="3" t="inlineStr">
         <is>
           <t>商用雷达、真实驾驶场景</t>
         </is>
       </c>
-      <c r="L34" s="3" t="inlineStr">
+      <c r="P34" s="3" t="inlineStr">
         <is>
           <t>任意距离/速度欺骗，抗多种计数器</t>
         </is>
       </c>
-      <c r="M34" s="3" t="inlineStr">
+      <c r="Q34" s="3" t="inlineStr">
         <is>
           <t>10.1109/SP46215.2023.10179371</t>
         </is>
       </c>
-      <c r="N34" s="3" t="inlineStr">
+      <c r="R34" s="3" t="inlineStr">
         <is>
           <t>无需与 victim 同步</t>
         </is>
@@ -2832,42 +3479,46 @@
           <t>定位与建图-在线高精地图</t>
         </is>
       </c>
-      <c r="G35" s="5" t="inlineStr">
+      <c r="G35" s="10" t="inlineStr"/>
+      <c r="H35" s="10" t="inlineStr"/>
+      <c r="I35" s="10" t="inlineStr"/>
+      <c r="J35" s="10" t="inlineStr"/>
+      <c r="K35" s="5" t="inlineStr">
         <is>
           <t>摄像头致盲 + 物理贴片（沿路线优化位置）</t>
         </is>
       </c>
-      <c r="H35" s="5" t="inlineStr">
+      <c r="L35" s="5" t="inlineStr">
         <is>
           <t>地图构建攻击</t>
         </is>
       </c>
-      <c r="I35" s="5" t="inlineStr">
+      <c r="M35" s="5" t="inlineStr">
         <is>
           <t>在线 HD map 构建模型（摘要未列名）</t>
         </is>
       </c>
-      <c r="J35" s="4" t="inlineStr">
+      <c r="N35" s="4" t="inlineStr">
         <is>
           <t>模型族</t>
         </is>
       </c>
-      <c r="K35" s="5" t="inlineStr">
+      <c r="O35" s="5" t="inlineStr">
         <is>
           <t>公开 AD 数据集 + 实车</t>
         </is>
       </c>
-      <c r="L35" s="5" t="inlineStr">
+      <c r="P35" s="5" t="inlineStr">
         <is>
           <t>建图精度最高 -9.9%，44% 路线不可达，不安全轨迹率最高 +27%</t>
         </is>
       </c>
-      <c r="M35" s="5" t="inlineStr">
+      <c r="Q35" s="5" t="inlineStr">
         <is>
           <t>10.1145/3719027.3765092</t>
         </is>
       </c>
-      <c r="N35" s="5" t="inlineStr">
+      <c r="R35" s="5" t="inlineStr">
         <is>
           <t>利用模型对对称道路结构的偏置</t>
         </is>
@@ -2900,42 +3551,46 @@
           <t>定位-无线室内定位</t>
         </is>
       </c>
-      <c r="G36" s="3" t="inlineStr">
+      <c r="G36" s="9" t="inlineStr"/>
+      <c r="H36" s="9" t="inlineStr"/>
+      <c r="I36" s="9" t="inlineStr"/>
+      <c r="J36" s="9" t="inlineStr"/>
+      <c r="K36" s="3" t="inlineStr">
         <is>
           <t>把场景中现有物体移动几厘米</t>
         </is>
       </c>
-      <c r="H36" s="3" t="inlineStr">
+      <c r="L36" s="3" t="inlineStr">
         <is>
           <t>物理物体摆放攻击</t>
         </is>
       </c>
-      <c r="I36" s="3" t="inlineStr">
+      <c r="M36" s="3" t="inlineStr">
         <is>
           <t>多种无线定位模型（摘要未列名）</t>
         </is>
       </c>
-      <c r="J36" s="2" t="inlineStr">
+      <c r="N36" s="2" t="inlineStr">
         <is>
           <t>模型族</t>
         </is>
       </c>
-      <c r="K36" s="3" t="inlineStr">
+      <c r="O36" s="3" t="inlineStr">
         <is>
           <t>真实室内场景</t>
         </is>
       </c>
-      <c r="L36" s="3" t="inlineStr">
+      <c r="P36" s="3" t="inlineStr">
         <is>
           <t>产生错误定位，跨模型/场景</t>
         </is>
       </c>
-      <c r="M36" s="3" t="inlineStr">
+      <c r="Q36" s="3" t="inlineStr">
         <is>
           <t>10.1109/TIFS.2025.3642536</t>
         </is>
       </c>
-      <c r="N36" s="3" t="inlineStr">
+      <c r="R36" s="3" t="inlineStr">
         <is>
           <t>可微射线追踪优化摆放</t>
         </is>
@@ -2968,42 +3623,46 @@
           <t>定位-WiFi 指纹定位</t>
         </is>
       </c>
-      <c r="G37" s="5" t="inlineStr">
+      <c r="G37" s="10" t="inlineStr"/>
+      <c r="H37" s="10" t="inlineStr"/>
+      <c r="I37" s="10" t="inlineStr"/>
+      <c r="J37" s="10" t="inlineStr"/>
+      <c r="K37" s="5" t="inlineStr">
         <is>
           <t>信号源端物理衰减噪声（Phy-Adv）</t>
         </is>
       </c>
-      <c r="H37" s="5" t="inlineStr">
+      <c r="L37" s="5" t="inlineStr">
         <is>
           <t>物理对抗样本</t>
         </is>
       </c>
-      <c r="I37" s="5" t="inlineStr">
+      <c r="M37" s="5" t="inlineStr">
         <is>
           <t>AlexNet、VGG、ResNet</t>
         </is>
       </c>
-      <c r="J37" s="4" t="inlineStr">
+      <c r="N37" s="4" t="inlineStr">
         <is>
           <t>具体型号</t>
         </is>
       </c>
-      <c r="K37" s="5" t="inlineStr">
+      <c r="O37" s="5" t="inlineStr">
         <is>
           <t>BHD、TUT 数据集</t>
         </is>
       </c>
-      <c r="L37" s="5" t="inlineStr">
+      <c r="P37" s="5" t="inlineStr">
         <is>
           <t>多模型有效；提出 RMBN 防御</t>
         </is>
       </c>
-      <c r="M37" s="5" t="inlineStr">
+      <c r="Q37" s="5" t="inlineStr">
         <is>
           <t>10.1109/TIFS.2024.3453041</t>
         </is>
       </c>
-      <c r="N37" s="5" t="inlineStr">
+      <c r="R37" s="5" t="inlineStr">
         <is>
           <t>从信号源端注入，而非改输入特征</t>
         </is>
@@ -3036,42 +3695,46 @@
           <t>定位/规划-UAV GNSS/IMU</t>
         </is>
       </c>
-      <c r="G38" s="3" t="inlineStr">
+      <c r="G38" s="9" t="inlineStr"/>
+      <c r="H38" s="9" t="inlineStr"/>
+      <c r="I38" s="9" t="inlineStr"/>
+      <c r="J38" s="9" t="inlineStr"/>
+      <c r="K38" s="3" t="inlineStr">
         <is>
           <t>GNSS 欺骗 + 运动状态触发后门</t>
         </is>
       </c>
-      <c r="H38" s="3" t="inlineStr">
+      <c r="L38" s="3" t="inlineStr">
         <is>
           <t>状态触发后门</t>
         </is>
       </c>
-      <c r="I38" s="3" t="inlineStr">
+      <c r="M38" s="3" t="inlineStr">
         <is>
           <t>GNSS/IMU 导航 + UAV 航路规划器（摘要未列名）；3 个检测器</t>
         </is>
       </c>
-      <c r="J38" s="2" t="inlineStr">
+      <c r="N38" s="2" t="inlineStr">
         <is>
           <t>模型族</t>
         </is>
       </c>
-      <c r="K38" s="3" t="inlineStr">
+      <c r="O38" s="3" t="inlineStr">
         <is>
           <t>UAV 航路规划仿真/实飞</t>
         </is>
       </c>
-      <c r="L38" s="3" t="inlineStr">
+      <c r="P38" s="3" t="inlineStr">
         <is>
           <t>定位误差显著增大、任务失败率高、检测器下高 stealth</t>
         </is>
       </c>
-      <c r="M38" s="3" t="inlineStr">
+      <c r="Q38" s="3" t="inlineStr">
         <is>
           <t>10.1109/TIFS.2025.3646036</t>
         </is>
       </c>
-      <c r="N38" s="3" t="inlineStr">
+      <c r="R38" s="3" t="inlineStr">
         <is>
           <t>把运动状态作为触发器</t>
         </is>
@@ -3104,42 +3767,46 @@
           <t>规划/控制-AD 系统</t>
         </is>
       </c>
-      <c r="G39" s="5" t="inlineStr">
+      <c r="G39" s="10" t="inlineStr"/>
+      <c r="H39" s="10" t="inlineStr"/>
+      <c r="I39" s="10" t="inlineStr"/>
+      <c r="J39" s="10" t="inlineStr"/>
+      <c r="K39" s="5" t="inlineStr">
         <is>
           <t>攻击车在交通中执行对抗性驾驶机动（场景级）</t>
         </is>
       </c>
-      <c r="H39" s="5" t="inlineStr">
+      <c r="L39" s="5" t="inlineStr">
         <is>
           <t>对抗驾驶机动搜索</t>
         </is>
       </c>
-      <c r="I39" s="5" t="inlineStr">
+      <c r="M39" s="5" t="inlineStr">
         <is>
           <t>openpilot、Autoware；CARLA</t>
         </is>
       </c>
-      <c r="J39" s="4" t="inlineStr">
+      <c r="N39" s="4" t="inlineStr">
         <is>
           <t>具体系统</t>
         </is>
       </c>
-      <c r="K39" s="5" t="inlineStr">
+      <c r="O39" s="5" t="inlineStr">
         <is>
           <t>CARLA 仿真</t>
         </is>
       </c>
-      <c r="L39" s="5" t="inlineStr">
+      <c r="P39" s="5" t="inlineStr">
         <is>
           <t>发现 341 次攻击（openpilot 219、Autoware 122），28 类</t>
         </is>
       </c>
-      <c r="M39" s="5" t="inlineStr">
+      <c r="Q39" s="5" t="inlineStr">
         <is>
           <t>https://www.usenix.org/conference/usenixsecurity23/presentation/song</t>
         </is>
       </c>
-      <c r="N39" s="5" t="inlineStr">
+      <c r="R39" s="5" t="inlineStr">
         <is>
           <t>不需要改传感器，只改交通行为</t>
         </is>
@@ -3172,42 +3839,46 @@
           <t>规划-轨迹预测</t>
         </is>
       </c>
-      <c r="G40" s="3" t="inlineStr">
+      <c r="G40" s="9" t="inlineStr"/>
+      <c r="H40" s="9" t="inlineStr"/>
+      <c r="I40" s="9" t="inlineStr"/>
+      <c r="J40" s="9" t="inlineStr"/>
+      <c r="K40" s="3" t="inlineStr">
         <is>
           <t>注入/篡改历史轨迹（Frenet 约束）</t>
         </is>
       </c>
-      <c r="H40" s="3" t="inlineStr">
+      <c r="L40" s="3" t="inlineStr">
         <is>
           <t>隐蔽对抗轨迹</t>
         </is>
       </c>
-      <c r="I40" s="3" t="inlineStr">
+      <c r="M40" s="3" t="inlineStr">
         <is>
           <t>2 个轨迹预测模型（摘要未列名）</t>
         </is>
       </c>
-      <c r="J40" s="2" t="inlineStr">
+      <c r="N40" s="2" t="inlineStr">
         <is>
           <t>模型族</t>
         </is>
       </c>
-      <c r="K40" s="3" t="inlineStr">
+      <c r="O40" s="3" t="inlineStr">
         <is>
           <t>2 个基准数据集 + 生产级仿真</t>
         </is>
       </c>
-      <c r="L40" s="3" t="inlineStr">
+      <c r="P40" s="3" t="inlineStr">
         <is>
           <t>ASR 超过 87%，可迁移、抗上游噪声</t>
         </is>
       </c>
-      <c r="M40" s="3" t="inlineStr">
+      <c r="Q40" s="3" t="inlineStr">
         <is>
           <t>10.1145/3705611</t>
         </is>
       </c>
-      <c r="N40" s="3" t="inlineStr">
+      <c r="R40" s="3" t="inlineStr">
         <is>
           <t>强调符合人类驾驶分布</t>
         </is>
@@ -3240,42 +3911,46 @@
           <t>协同/决策-多智能体强化学习</t>
         </is>
       </c>
-      <c r="G41" s="5" t="inlineStr">
+      <c r="G41" s="10" t="inlineStr"/>
+      <c r="H41" s="10" t="inlineStr"/>
+      <c r="I41" s="10" t="inlineStr"/>
+      <c r="J41" s="10" t="inlineStr"/>
+      <c r="K41" s="5" t="inlineStr">
         <is>
           <t>控制部分对手智能体，黑盒策略交互</t>
         </is>
       </c>
-      <c r="H41" s="5" t="inlineStr">
+      <c r="L41" s="5" t="inlineStr">
         <is>
           <t>部分可观测对抗策略</t>
         </is>
       </c>
-      <c r="I41" s="5" t="inlineStr">
+      <c r="M41" s="5" t="inlineStr">
         <is>
           <t>DDPG、MADDPG（实验）；QMIX、MAPPO（算法无关性讨论）；Predator-prey、World Communication</t>
         </is>
       </c>
-      <c r="J41" s="4" t="inlineStr">
+      <c r="N41" s="4" t="inlineStr">
         <is>
           <t>具体算法</t>
         </is>
       </c>
-      <c r="K41" s="5" t="inlineStr">
+      <c r="O41" s="5" t="inlineStr">
         <is>
           <t>两个多智能体竞争环境</t>
         </is>
       </c>
-      <c r="L41" s="5" t="inlineStr">
+      <c r="P41" s="5" t="inlineStr">
         <is>
           <t>78%/80% 场景优于基线；可用于无人机集群</t>
         </is>
       </c>
-      <c r="M41" s="5" t="inlineStr">
+      <c r="Q41" s="5" t="inlineStr">
         <is>
           <t>10.1145/3658644.3670293</t>
         </is>
       </c>
-      <c r="N41" s="5" t="inlineStr">
+      <c r="R41" s="5" t="inlineStr">
         <is>
           <t>面向部分可观测多智能体系统</t>
         </is>
@@ -3308,42 +3983,62 @@
           <t>感知/导航-扫地机器人</t>
         </is>
       </c>
-      <c r="G42" s="3" t="inlineStr">
+      <c r="G42" s="9" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="H42" s="9" t="inlineStr">
+        <is>
+          <t>相机 / 视觉传感器</t>
+        </is>
+      </c>
+      <c r="I42" s="9" t="inlineStr">
+        <is>
+          <t>T1c</t>
+        </is>
+      </c>
+      <c r="J42" s="9" t="inlineStr">
+        <is>
+          <t>多视角/机器人视觉</t>
+        </is>
+      </c>
+      <c r="K42" s="3" t="inlineStr">
         <is>
           <t>地面视角对抗贴片（GPatch）</t>
         </is>
       </c>
-      <c r="H42" s="3" t="inlineStr">
+      <c r="L42" s="3" t="inlineStr">
         <is>
           <t>隐私保护型对抗补丁（阻止进入）</t>
         </is>
       </c>
-      <c r="I42" s="3" t="inlineStr">
+      <c r="M42" s="3" t="inlineStr">
         <is>
           <t>相机-based RVC 导航/决策（摘要未列名）</t>
         </is>
       </c>
-      <c r="J42" s="2" t="inlineStr">
+      <c r="N42" s="2" t="inlineStr">
         <is>
           <t>模型族</t>
         </is>
       </c>
-      <c r="K42" s="3" t="inlineStr">
+      <c r="O42" s="3" t="inlineStr">
         <is>
           <t>真实家庭环境</t>
         </is>
       </c>
-      <c r="L42" s="3" t="inlineStr">
+      <c r="P42" s="3" t="inlineStr">
         <is>
           <t>平均 87.27% 阻止进入成功率</t>
         </is>
       </c>
-      <c r="M42" s="3" t="inlineStr">
+      <c r="Q42" s="3" t="inlineStr">
         <is>
           <t>10.1109/TDSC.2025.3603988</t>
         </is>
       </c>
-      <c r="N42" s="3" t="inlineStr">
+      <c r="R42" s="3" t="inlineStr">
         <is>
           <t>防御性对抗样本，但接入方式可复用</t>
         </is>
@@ -3376,42 +4071,46 @@
           <t>全链路（体系化）</t>
         </is>
       </c>
-      <c r="G43" s="5" t="inlineStr">
+      <c r="G43" s="10" t="inlineStr"/>
+      <c r="H43" s="10" t="inlineStr"/>
+      <c r="I43" s="10" t="inlineStr"/>
+      <c r="J43" s="10" t="inlineStr"/>
+      <c r="K43" s="5" t="inlineStr">
         <is>
           <t>7 类传感器欺骗攻击路径</t>
         </is>
       </c>
-      <c r="H43" s="5" t="inlineStr">
+      <c r="L43" s="5" t="inlineStr">
         <is>
           <t>SoK/分类体系</t>
         </is>
       </c>
-      <c r="I43" s="5" t="inlineStr">
+      <c r="M43" s="5" t="inlineStr">
         <is>
           <t>机器人车辆感知、定位、控制</t>
         </is>
       </c>
-      <c r="J43" s="4" t="inlineStr">
+      <c r="N43" s="4" t="inlineStr">
         <is>
           <t>系统级</t>
         </is>
       </c>
-      <c r="K43" s="5" t="inlineStr">
+      <c r="O43" s="5" t="inlineStr">
         <is>
           <t>文献系统化</t>
         </is>
       </c>
-      <c r="L43" s="5" t="inlineStr">
+      <c r="P43" s="5" t="inlineStr">
         <is>
           <t>识别攻击路径与未探索空白</t>
         </is>
       </c>
-      <c r="M43" s="5" t="inlineStr">
+      <c r="Q43" s="5" t="inlineStr">
         <is>
           <t>10.1109/EuroSP57164.2023.00067</t>
         </is>
       </c>
-      <c r="N43" s="5" t="inlineStr">
+      <c r="R43" s="5" t="inlineStr">
         <is>
           <t>适合作为接入手段分类框架</t>
         </is>
@@ -3444,42 +4143,46 @@
           <t>全链路（测量）</t>
         </is>
       </c>
-      <c r="G44" s="3" t="inlineStr">
+      <c r="G44" s="9" t="inlineStr"/>
+      <c r="H44" s="9" t="inlineStr"/>
+      <c r="I44" s="9" t="inlineStr"/>
+      <c r="J44" s="9" t="inlineStr"/>
+      <c r="K44" s="3" t="inlineStr">
         <is>
           <t>物理传感器攻击难度测量</t>
         </is>
       </c>
-      <c r="H44" s="3" t="inlineStr">
+      <c r="L44" s="3" t="inlineStr">
         <is>
           <t>测量研究</t>
         </is>
       </c>
-      <c r="I44" s="3" t="inlineStr">
+      <c r="M44" s="3" t="inlineStr">
         <is>
           <t>机器人/无人系统传感器</t>
         </is>
       </c>
-      <c r="J44" s="2" t="inlineStr">
+      <c r="N44" s="2" t="inlineStr">
         <is>
           <t>系统级</t>
         </is>
       </c>
-      <c r="K44" s="3" t="inlineStr">
+      <c r="O44" s="3" t="inlineStr">
         <is>
           <t>多类传感器/系统</t>
         </is>
       </c>
-      <c r="L44" s="3" t="inlineStr">
+      <c r="P44" s="3" t="inlineStr">
         <is>
           <t>提出攻击硬度评估框架</t>
         </is>
       </c>
-      <c r="M44" s="3" t="inlineStr">
+      <c r="Q44" s="3" t="inlineStr">
         <is>
           <t>10.1109/SP54263.2024.00143</t>
         </is>
       </c>
-      <c r="N44" s="3" t="inlineStr">
+      <c r="R44" s="3" t="inlineStr">
         <is>
           <t>可用于评估接入可行性</t>
         </is>
@@ -3512,42 +4215,62 @@
           <t>感知-相机 2D 检测 + 车道线检测</t>
         </is>
       </c>
-      <c r="G45" s="5" t="inlineStr">
+      <c r="G45" s="10" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="H45" s="10" t="inlineStr">
+        <is>
+          <t>相机 / 视觉传感器</t>
+        </is>
+      </c>
+      <c r="I45" s="10" t="inlineStr">
+        <is>
+          <t>T1d</t>
+        </is>
+      </c>
+      <c r="J45" s="10" t="inlineStr">
+        <is>
+          <t>相机信号注入</t>
+        </is>
+      </c>
+      <c r="K45" s="5" t="inlineStr">
         <is>
           <t>声学信号操纵相机防抖 IMU，诱发图像模糊</t>
         </is>
       </c>
-      <c r="H45" s="5" t="inlineStr">
+      <c r="L45" s="5" t="inlineStr">
         <is>
           <t>系统级物理对抗/致盲</t>
         </is>
       </c>
-      <c r="I45" s="5" t="inlineStr">
+      <c r="M45" s="5" t="inlineStr">
         <is>
           <t>YOLOv3/v4/v5、Faster R-CNN、Apollo、UFLD、LaneAF</t>
         </is>
       </c>
-      <c r="J45" s="4" t="inlineStr">
+      <c r="N45" s="4" t="inlineStr">
         <is>
           <t>具体型号</t>
         </is>
       </c>
-      <c r="K45" s="5" t="inlineStr">
+      <c r="O45" s="5" t="inlineStr">
         <is>
           <t>真实相机/车载场景</t>
         </is>
       </c>
-      <c r="L45" s="5" t="inlineStr">
+      <c r="P45" s="5" t="inlineStr">
         <is>
           <t>隐藏/创建/改变三类攻击；5 个检测器 + 2 个车道线检测器均受影响</t>
         </is>
       </c>
-      <c r="M45" s="5" t="inlineStr">
+      <c r="Q45" s="5" t="inlineStr">
         <is>
           <t>10.1109/TDSC.2023.3334618</t>
         </is>
       </c>
-      <c r="N45" s="5" t="inlineStr">
+      <c r="R45" s="5" t="inlineStr">
         <is>
           <t>AMpLe；声学触发直接作用于防抖传感器，与 TPatch 的相机畸变路径不同</t>
         </is>
@@ -3580,42 +4303,62 @@
           <t>感知-相机 2D 分类/检测</t>
         </is>
       </c>
-      <c r="G46" s="3" t="inlineStr">
+      <c r="G46" s="9" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="H46" s="9" t="inlineStr">
+        <is>
+          <t>相机 / 视觉传感器</t>
+        </is>
+      </c>
+      <c r="I46" s="9" t="inlineStr">
+        <is>
+          <t>T1d</t>
+        </is>
+      </c>
+      <c r="J46" s="9" t="inlineStr">
+        <is>
+          <t>相机信号注入</t>
+        </is>
+      </c>
+      <c r="K46" s="3" t="inlineStr">
         <is>
           <t>低成本便携设备注入电磁信号，直接操纵 CCD 图像输出</t>
         </is>
       </c>
-      <c r="H46" s="3" t="inlineStr">
+      <c r="L46" s="3" t="inlineStr">
         <is>
           <t>物理对抗样本（无接触/无可见贴片）</t>
         </is>
       </c>
-      <c r="I46" s="3" t="inlineStr">
+      <c r="M46" s="3" t="inlineStr">
         <is>
           <t>Inception-v3、ResNet-101、YOLOv3/v4</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr">
+      <c r="N46" s="2" t="inlineStr">
         <is>
           <t>具体型号</t>
         </is>
       </c>
-      <c r="K46" s="3" t="inlineStr">
+      <c r="O46" s="3" t="inlineStr">
         <is>
           <t>5 款相机、真实场景</t>
         </is>
       </c>
-      <c r="L46" s="3" t="inlineStr">
+      <c r="P46" s="3" t="inlineStr">
         <is>
           <t>无目标/有目标/隐藏/出现四类攻击；跨 5 款相机和多个 DNN 有效</t>
         </is>
       </c>
-      <c r="M46" s="3" t="inlineStr">
+      <c r="Q46" s="3" t="inlineStr">
         <is>
           <t>10.1109/TDSC.2025.3529197</t>
         </is>
       </c>
-      <c r="N46" s="3" t="inlineStr">
+      <c r="R46" s="3" t="inlineStr">
         <is>
           <t>不需要接触目标物体，接入点是相机传感器</t>
         </is>
@@ -3648,42 +4391,62 @@
           <t>感知-交通标志识别</t>
         </is>
       </c>
-      <c r="G47" s="5" t="inlineStr">
+      <c r="G47" s="10" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="H47" s="10" t="inlineStr">
+        <is>
+          <t>相机 / 视觉传感器</t>
+        </is>
+      </c>
+      <c r="I47" s="10" t="inlineStr">
+        <is>
+          <t>T1b</t>
+        </is>
+      </c>
+      <c r="J47" s="10" t="inlineStr">
+        <is>
+          <t>交通标志专用视觉</t>
+        </is>
+      </c>
+      <c r="K47" s="5" t="inlineStr">
         <is>
           <t>把自然磨损/老化纹理作为对抗载体（GAN 损伤风格编码 + 扰动）</t>
         </is>
       </c>
-      <c r="H47" s="5" t="inlineStr">
+      <c r="L47" s="5" t="inlineStr">
         <is>
           <t>自然化物理对抗样本</t>
         </is>
       </c>
-      <c r="I47" s="5" t="inlineStr">
+      <c r="M47" s="5" t="inlineStr">
         <is>
           <t>交通标志识别 DNN（摘要未列具体型号）</t>
         </is>
       </c>
-      <c r="J47" s="4" t="inlineStr">
+      <c r="N47" s="4" t="inlineStr">
         <is>
           <t>模型族</t>
         </is>
       </c>
-      <c r="K47" s="5" t="inlineStr">
+      <c r="O47" s="5" t="inlineStr">
         <is>
           <t>两个交通标志数据集；数字 + 物理</t>
         </is>
       </c>
-      <c r="L47" s="5" t="inlineStr">
+      <c r="P47" s="5" t="inlineStr">
         <is>
           <t>有效 ASR、跨模型迁移、自然外观；训练时可增强真实损伤泛化</t>
         </is>
       </c>
-      <c r="M47" s="5" t="inlineStr">
+      <c r="Q47" s="5" t="inlineStr">
         <is>
           <t>10.1109/TDSC.2026.3660107</t>
         </is>
       </c>
-      <c r="N47" s="5" t="inlineStr">
+      <c r="R47" s="5" t="inlineStr">
         <is>
           <t>AdvWT；代码已开源；把自然损坏变成物理接入</t>
         </is>
@@ -3716,42 +4479,62 @@
           <t>感知-视觉单目标跟踪</t>
         </is>
       </c>
-      <c r="G48" s="3" t="inlineStr">
+      <c r="G48" s="9" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="H48" s="9" t="inlineStr">
+        <is>
+          <t>感知算法 / 数据层</t>
+        </is>
+      </c>
+      <c r="I48" s="9" t="inlineStr">
+        <is>
+          <t>T4b</t>
+        </is>
+      </c>
+      <c r="J48" s="9" t="inlineStr">
+        <is>
+          <t>视觉单目标跟踪</t>
+        </is>
+      </c>
+      <c r="K48" s="3" t="inlineStr">
         <is>
           <t>决策式黑盒查询；按图像块压缩对抗噪声</t>
         </is>
       </c>
-      <c r="H48" s="3" t="inlineStr">
+      <c r="L48" s="3" t="inlineStr">
         <is>
           <t>块级噪声压缩攻击（PANC）</t>
         </is>
       </c>
-      <c r="I48" s="3" t="inlineStr">
+      <c r="M48" s="3" t="inlineStr">
         <is>
           <t>OSTrack、STARK、TransT、MixFormerV2</t>
         </is>
       </c>
-      <c r="J48" s="2" t="inlineStr">
+      <c r="N48" s="2" t="inlineStr">
         <is>
           <t>具体型号</t>
         </is>
       </c>
-      <c r="K48" s="3" t="inlineStr">
+      <c r="O48" s="3" t="inlineStr">
         <is>
           <t>GOT-10k、TrackingNet、LaSOT</t>
         </is>
       </c>
-      <c r="L48" s="3" t="inlineStr">
+      <c r="P48" s="3" t="inlineStr">
         <is>
           <t>噪声压缩到 10%，攻击效果相对 IoU attack +162%，查询量 45.7%</t>
         </is>
       </c>
-      <c r="M48" s="3" t="inlineStr">
+      <c r="Q48" s="3" t="inlineStr">
         <is>
           <t>10.1109/TIFS.2025.3648551</t>
         </is>
       </c>
-      <c r="N48" s="3" t="inlineStr">
+      <c r="R48" s="3" t="inlineStr">
         <is>
           <t>补上 Transformer 跟踪器；与 Siam 系跟踪攻击互补</t>
         </is>
@@ -3784,42 +4567,62 @@
           <t>感知-LiDAR 3D 检测</t>
         </is>
       </c>
-      <c r="G49" s="5" t="inlineStr">
+      <c r="G49" s="10" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="H49" s="10" t="inlineStr">
+        <is>
+          <t>LiDAR / 点云传感器</t>
+        </is>
+      </c>
+      <c r="I49" s="10" t="inlineStr">
+        <is>
+          <t>T2c</t>
+        </is>
+      </c>
+      <c r="J49" s="10" t="inlineStr">
+        <is>
+          <t>跨模态/多传感器融合</t>
+        </is>
+      </c>
+      <c r="K49" s="5" t="inlineStr">
         <is>
           <t>IEMI 电磁干扰注入 LiDAR 接收/监测/光束控制模块</t>
         </is>
       </c>
-      <c r="H49" s="5" t="inlineStr">
+      <c r="L49" s="5" t="inlineStr">
         <is>
           <t>跨模态信号注入（点云干扰/注入/删除/断电）</t>
         </is>
       </c>
-      <c r="I49" s="5" t="inlineStr">
+      <c r="M49" s="5" t="inlineStr">
         <is>
           <t>PointPillar、PV-RCNN、VirConv-L、EPNet、CLOCs</t>
         </is>
       </c>
-      <c r="J49" s="4" t="inlineStr">
+      <c r="N49" s="4" t="inlineStr">
         <is>
           <t>具体型号</t>
         </is>
       </c>
-      <c r="K49" s="5" t="inlineStr">
+      <c r="O49" s="5" t="inlineStr">
         <is>
           <t>5 款 COTS LiDAR；仿真 + 真实 + 移动场景</t>
         </is>
       </c>
-      <c r="L49" s="5" t="inlineStr">
+      <c r="P49" s="5" t="inlineStr">
         <is>
           <t>点云干扰/注入/删除，甚至 LiDAR 断电；跨检测与融合模型</t>
         </is>
       </c>
-      <c r="M49" s="5" t="inlineStr">
+      <c r="Q49" s="5" t="inlineStr">
         <is>
           <t>10.14722/ndss.2025.230997</t>
         </is>
       </c>
-      <c r="N49" s="5" t="inlineStr">
+      <c r="R49" s="5" t="inlineStr">
         <is>
           <t>接入点从激光转到电磁侧信道；可绕过纯光学防御</t>
         </is>
@@ -3852,42 +4655,46 @@
           <t>规划/决策-ADS 决策模块</t>
         </is>
       </c>
-      <c r="G50" s="3" t="inlineStr">
+      <c r="G50" s="9" t="inlineStr"/>
+      <c r="H50" s="9" t="inlineStr"/>
+      <c r="I50" s="9" t="inlineStr"/>
+      <c r="J50" s="9" t="inlineStr"/>
+      <c r="K50" s="3" t="inlineStr">
         <is>
           <t>控制多辆交通车执行直接/间接多车对抗行为</t>
         </is>
       </c>
-      <c r="H50" s="3" t="inlineStr">
+      <c r="L50" s="3" t="inlineStr">
         <is>
           <t>多车场景级对抗行为（LLM + 遗传算法搜索）</t>
         </is>
       </c>
-      <c r="I50" s="3" t="inlineStr">
+      <c r="M50" s="3" t="inlineStr">
         <is>
           <t>Baidu Apollo ADS / Apollo 6.0（Waymo 为背景系统）</t>
         </is>
       </c>
-      <c r="J50" s="2" t="inlineStr">
+      <c r="N50" s="2" t="inlineStr">
         <is>
           <t>具体系统</t>
         </is>
       </c>
-      <c r="K50" s="3" t="inlineStr">
+      <c r="O50" s="3" t="inlineStr">
         <is>
           <t>真实事故报告 + Apollo 仿真 + 2 辆 Apollo 6.0 实车</t>
         </is>
       </c>
-      <c r="L50" s="3" t="inlineStr">
+      <c r="P50" s="3" t="inlineStr">
         <is>
           <t>发现 14 类攻击模式，实车验证多车攻击可行性</t>
         </is>
       </c>
-      <c r="M50" s="3" t="inlineStr">
+      <c r="Q50" s="3" t="inlineStr">
         <is>
           <t>10.1109/TDSC.2026.3741897</t>
         </is>
       </c>
-      <c r="N50" s="3" t="inlineStr">
+      <c r="R50" s="3" t="inlineStr">
         <is>
           <t>Tracking 方法；从人类事故中挖掘攻击先验</t>
         </is>
@@ -3920,42 +4727,62 @@
           <t>感知-2D 目标检测（行人）</t>
         </is>
       </c>
-      <c r="G51" s="5" t="inlineStr">
+      <c r="G51" s="10" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="H51" s="10" t="inlineStr">
+        <is>
+          <t>相机 / 视觉传感器</t>
+        </is>
+      </c>
+      <c r="I51" s="10" t="inlineStr">
+        <is>
+          <t>T1a</t>
+        </is>
+      </c>
+      <c r="J51" s="10" t="inlineStr">
+        <is>
+          <t>单目 2D 检测/分类</t>
+        </is>
+      </c>
+      <c r="K51" s="5" t="inlineStr">
         <is>
           <t>打印在衣物上的对抗图案/贴片</t>
         </is>
       </c>
-      <c r="H51" s="5" t="inlineStr">
+      <c r="L51" s="5" t="inlineStr">
         <is>
           <t>动态集成物理补丁</t>
         </is>
       </c>
-      <c r="I51" s="5" t="inlineStr">
+      <c r="M51" s="5" t="inlineStr">
         <is>
           <t>YOLOv2、YOLOv3；5 个主流检测器</t>
         </is>
       </c>
-      <c r="J51" s="4" t="inlineStr">
+      <c r="N51" s="4" t="inlineStr">
         <is>
           <t>具体型号</t>
         </is>
       </c>
-      <c r="K51" s="5" t="inlineStr">
+      <c r="O51" s="5" t="inlineStr">
         <is>
           <t>数字 + 物理 T 恤</t>
         </is>
       </c>
-      <c r="L51" s="5" t="inlineStr">
+      <c r="P51" s="5" t="inlineStr">
         <is>
           <t>YOLOv2/YOLOv3 识别率降至 13.19%/29.20%</t>
         </is>
       </c>
-      <c r="M51" s="5" t="inlineStr">
+      <c r="Q51" s="5" t="inlineStr">
         <is>
           <t>10.1109/TIFS.2024.3468908</t>
         </is>
       </c>
-      <c r="N51" s="5" t="inlineStr">
+      <c r="R51" s="5" t="inlineStr">
         <is>
           <t>黑盒集成 + 能量优化；可迁移到人体/机器人目标检测</t>
         </is>
@@ -3988,42 +4815,46 @@
           <t>全链路-无人车/UxV 攻击面</t>
         </is>
       </c>
-      <c r="G52" s="3" t="inlineStr">
+      <c r="G52" s="9" t="inlineStr"/>
+      <c r="H52" s="9" t="inlineStr"/>
+      <c r="I52" s="9" t="inlineStr"/>
+      <c r="J52" s="9" t="inlineStr"/>
+      <c r="K52" s="3" t="inlineStr">
         <is>
           <t>系统化分类（感知/通信/控制/供应链等）</t>
         </is>
       </c>
-      <c r="H52" s="3" t="inlineStr">
+      <c r="L52" s="3" t="inlineStr">
         <is>
           <t>SoK/系统分类</t>
         </is>
       </c>
-      <c r="I52" s="3" t="inlineStr">
+      <c r="M52" s="3" t="inlineStr">
         <is>
           <t>无人车/UxV 系统组件</t>
         </is>
       </c>
-      <c r="J52" s="2" t="inlineStr">
+      <c r="N52" s="2" t="inlineStr">
         <is>
           <t>系统级</t>
         </is>
       </c>
-      <c r="K52" s="3" t="inlineStr">
+      <c r="O52" s="3" t="inlineStr">
         <is>
           <t>文献系统化</t>
         </is>
       </c>
-      <c r="L52" s="3" t="inlineStr">
+      <c r="P52" s="3" t="inlineStr">
         <is>
           <t>给出 UxV 攻击面与防御研究议程</t>
         </is>
       </c>
-      <c r="M52" s="3" t="inlineStr">
+      <c r="Q52" s="3" t="inlineStr">
         <is>
           <t>10.1109/EuroSP68448.2026.00031</t>
         </is>
       </c>
-      <c r="N52" s="3" t="inlineStr">
+      <c r="R52" s="3" t="inlineStr">
         <is>
           <t>2026 年新增 SoK；用于校核阶段划分</t>
         </is>
@@ -4056,42 +4887,46 @@
           <t>体系化-相机图像处理流水线</t>
         </is>
       </c>
-      <c r="G53" s="5" t="inlineStr">
+      <c r="G53" s="10" t="inlineStr"/>
+      <c r="H53" s="10" t="inlineStr"/>
+      <c r="I53" s="10" t="inlineStr"/>
+      <c r="J53" s="10" t="inlineStr"/>
+      <c r="K53" s="5" t="inlineStr">
         <is>
           <t>按图像处理 pipeline 分层分析攻击接入</t>
         </is>
       </c>
-      <c r="H53" s="5" t="inlineStr">
+      <c r="L53" s="5" t="inlineStr">
         <is>
           <t>SoK/系统分类</t>
         </is>
       </c>
-      <c r="I53" s="5" t="inlineStr">
+      <c r="M53" s="5" t="inlineStr">
         <is>
           <t>相机感知 pipeline（92 篇文献）</t>
         </is>
       </c>
-      <c r="J53" s="4" t="inlineStr">
+      <c r="N53" s="4" t="inlineStr">
         <is>
           <t>系统级</t>
         </is>
       </c>
-      <c r="K53" s="5" t="inlineStr">
+      <c r="O53" s="5" t="inlineStr">
         <is>
           <t>文献系统化 + ISO 21434 + PICT testbed</t>
         </is>
       </c>
-      <c r="L53" s="5" t="inlineStr">
+      <c r="P53" s="5" t="inlineStr">
         <is>
           <t>把攻击面拆到镜头/ISP/传输/模型多层</t>
         </is>
       </c>
-      <c r="M53" s="5" t="inlineStr">
+      <c r="Q53" s="5" t="inlineStr">
         <is>
           <t>10.1145/3779208.3785267</t>
         </is>
       </c>
-      <c r="N53" s="5" t="inlineStr">
+      <c r="R53" s="5" t="inlineStr">
         <is>
           <t>补足相机链路内部接入层；TARA-CAM 工具</t>
         </is>
@@ -4124,55 +4959,662 @@
           <t>感知-相机 2D 检测 + ACC 控制</t>
         </is>
       </c>
-      <c r="G54" s="3" t="inlineStr">
+      <c r="G54" s="9" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="H54" s="9" t="inlineStr">
+        <is>
+          <t>感知算法 / 数据层</t>
+        </is>
+      </c>
+      <c r="I54" s="9" t="inlineStr">
+        <is>
+          <t>T4d</t>
+        </is>
+      </c>
+      <c r="J54" s="9" t="inlineStr">
+        <is>
+          <t>运行时 ACC 链路</t>
+        </is>
+      </c>
+      <c r="K54" s="3" t="inlineStr">
         <is>
           <t>运行时向相机数据注入对抗扰动；按场景选择触发时机</t>
         </is>
       </c>
-      <c r="H54" s="3" t="inlineStr">
+      <c r="L54" s="3" t="inlineStr">
         <is>
           <t>上下文触发式运行时感知攻击</t>
         </is>
       </c>
-      <c r="I54" s="3" t="inlineStr">
+      <c r="M54" s="3" t="inlineStr">
         <is>
           <t>DNN-based ACC 感知/控制模型；生产级 ACC 控制软件；AEBS 安全机制</t>
         </is>
       </c>
-      <c r="J54" s="2" t="inlineStr">
+      <c r="N54" s="2" t="inlineStr">
         <is>
           <t>模型族</t>
         </is>
       </c>
-      <c r="K54" s="3" t="inlineStr">
+      <c r="O54" s="3" t="inlineStr">
         <is>
           <t>实车 + 公开驾驶数据集 + 生产级 ACC 仿真 + 驾驶模拟器</t>
         </is>
       </c>
-      <c r="L54" s="3" t="inlineStr">
+      <c r="P54" s="3" t="inlineStr">
         <is>
           <t>造成危险的攻击成功率较基线高 142.9 倍；规避率提升 82.6%</t>
         </is>
       </c>
-      <c r="M54" s="3" t="inlineStr">
+      <c r="Q54" s="3" t="inlineStr">
         <is>
           <t>10.1145/3708821.3710832</t>
         </is>
       </c>
-      <c r="N54" s="3" t="inlineStr">
+      <c r="R54" s="3" t="inlineStr">
         <is>
           <t>把相机扰动接到 ACC 控制闭环，并评估驾驶员接管与 AEBS；补足控制耦合证据</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N54"/>
+  <autoFilter ref="A1:R54"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="62" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>攻击目标代码</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>攻击目标</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>层级</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>算法分支代码</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>算法分支</t>
+        </is>
+      </c>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t>说明</t>
+        </is>
+      </c>
+      <c r="G1" s="11" t="inlineStr">
+        <is>
+          <t>论文数</t>
+        </is>
+      </c>
+      <c r="H1" s="11" t="inlineStr">
+        <is>
+          <t>论文ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>相机 / 视觉传感器</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>传感器层</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>T1a</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>单目 2D 检测/分类</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>面向普通单目相机图像的单阶段 2D 检测、分类、多目标跟踪与 NMS 后处理链路。</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="H2" s="7" t="inlineStr">
+        <is>
+          <t>1、2、3、12、30、50</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>相机 / 视觉传感器</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>传感器层</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>T1b</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>交通标志专用视觉</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>面向交通标志检测、识别与商用 TSR 的专用视觉任务，含贴片、投影、近红外与自然损伤。</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>6、7、8、9、11、46</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>相机 / 视觉传感器</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>传感器层</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>T1c</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>多视角/机器人视觉</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>多视角/环视相机中的 3D 视觉对抗物体，以及扫地机器人地视角导航的隐私保护型攻击。</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>24、41</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>相机 / 视觉传感器</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>传感器层</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>T1d</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>相机信号注入</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>通过声学或电磁信号改写相机成像链路，重点不在可见贴片，而在传感器信号与图像畸变。</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>44、45</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>LiDAR / 点云传感器</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>传感器层</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>T2a</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>LiDAR 3D 检测</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>面向 PointPillars、PointRCNN、SECOND、PV-RCNN 等 LiDAR 3D 检测器的注入、移除与对抗物体攻击。</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>17、18、19、21、22</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>LiDAR / 点云传感器</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>传感器层</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>T2b</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>点云欺骗/闭环验证</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>反射率欺骗、长时点云伪造及规划控制闭环验证，强调物理可实现性与系统级后果。</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>20、23</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>LiDAR / 点云传感器</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>传感器层</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>T2c</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>跨模态/多传感器融合</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>视觉与 LiDAR 联合的跨模态对抗物体，以及针对融合感知链路的跨模态信号注入。</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>25、48</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>毫米波雷达传感器</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>传感器层</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>T3a</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>学习型雷达检测</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>以 DNN 雷达目标检测模型为直接对象的被动反射对抗物体攻击。</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>毫米波雷达传感器</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>传感器层</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>T3b</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>FMCW 信号层</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>直接操纵 FMCW 雷达波形、距离与速度估计的物理层欺骗，不依赖学习型检测器。</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>32、33</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>感知算法 / 数据层</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>算法与数据层</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>T4a</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>点云分类与预处理</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>点云语义分类、硬标签黑盒、后门投毒、形变扰动与 LiDAR 预处理层攻击。</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>26、27、28、29</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>感知算法 / 数据层</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>算法与数据层</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>T4b</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>视觉单目标跟踪</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>面向 DCF、Siamese、Transformer 与 OSTrack 类视觉跟踪器的轨迹劫持和特征级攻击。</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>15、16、47</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>感知算法 / 数据层</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>算法与数据层</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>T4c</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>单目深度/后门</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>单目深度估计的物理透视劫持，以及交通标志检测中的物理后门与数据投毒。</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>4、10</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>感知算法 / 数据层</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>算法与数据层</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>T4d</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>运行时 ACC 链路</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>面向 DNN 感知与自适应巡航控制链路的上下文触发式运行时感知攻击。</t>
+        </is>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H14"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4225,7 +5667,7 @@
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>相机/LiDAR/点云/雷达/深度/跟踪，攻击面最成熟</t>
+          <t>相机/LiDAR/点云/雷达/深度/跟踪，攻击面最成熟；现已细分为 4 个攻击目标、13 个算法分支</t>
         </is>
       </c>
     </row>
@@ -4294,7 +5736,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4842,13 +6284,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5011,18 +6453,30 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>S1 分类口径</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>S1 先按攻击目标拆为 T1—T4，再按论文任务与模型字段拆为 13 个算法分支；非 S1 行的目标与分支字段留空。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5149,6 +6603,18 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>S1 分类复核</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>38 篇感知论文全部映射至 4 个攻击目标、13 个算法分支；无遗漏、无重复。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>